<commit_message>
feat: add image compression
</commit_message>
<xml_diff>
--- a/src/locales/moneyGone.xlsx
+++ b/src/locales/moneyGone.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="480">
   <si>
     <t>key</t>
   </si>
@@ -896,6 +896,21 @@
   </si>
   <si>
     <t>画像のサイズは2MBを超えてはいけません</t>
+  </si>
+  <si>
+    <t>LC_IMG_UPLOAD_ERROR</t>
+  </si>
+  <si>
+    <t>圖片上傳失敗</t>
+  </si>
+  <si>
+    <t>图片上传失败</t>
+  </si>
+  <si>
+    <t>Image upload failed</t>
+  </si>
+  <si>
+    <t>画像のアップロードに失敗しました</t>
   </si>
   <si>
     <t>LC_CATEGORY_DELETE</t>
@@ -2820,28 +2835,28 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1"/>
-      <c r="B70" s="1"/>
-      <c r="C70" s="1"/>
-      <c r="D70" s="1"/>
-      <c r="E70" s="1"/>
+      <c r="A70" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>314</v>
-      </c>
+      <c r="A71" s="1"/>
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
@@ -3014,28 +3029,28 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1"/>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
+      <c r="A82" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>369</v>
-      </c>
+      <c r="A83" s="1"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="s">
@@ -3157,28 +3172,28 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1"/>
-      <c r="B91" s="1"/>
-      <c r="C91" s="1"/>
-      <c r="D91" s="1"/>
-      <c r="E91" s="1"/>
+      <c r="A91" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>409</v>
-      </c>
+      <c r="A92" s="1"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="s">
@@ -3198,28 +3213,28 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1"/>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-      <c r="D94" s="1"/>
-      <c r="E94" s="1"/>
+      <c r="A94" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="D95" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>419</v>
-      </c>
+      <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="s">
@@ -3256,28 +3271,28 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1"/>
-      <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
-      <c r="D98" s="1"/>
-      <c r="E98" s="1"/>
+      <c r="A98" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>434</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>434</v>
-      </c>
+      <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="s">
@@ -3304,71 +3319,71 @@
         <v>441</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1"/>
-      <c r="B103" s="1"/>
-      <c r="C103" s="1"/>
-      <c r="D103" s="1"/>
-      <c r="E103" s="1"/>
+      <c r="A103" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>452</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="D104" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>449</v>
-      </c>
+      <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D105" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="E105" s="1" t="s">
         <v>454</v>
-      </c>
-      <c r="E105" s="1" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="106">
@@ -3379,21 +3394,21 @@
         <v>457</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>462</v>
@@ -3437,6 +3452,23 @@
       </c>
       <c r="E109" s="1" t="s">
         <v>474</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: adjust lang, style
</commit_message>
<xml_diff>
--- a/src/locales/moneyGone.xlsx
+++ b/src/locales/moneyGone.xlsx
@@ -106,7 +106,7 @@
     <t>剩余</t>
   </si>
   <si>
-    <t>Remaining</t>
+    <t>Left</t>
   </si>
   <si>
     <t>残り</t>
@@ -466,10 +466,10 @@
     <t>月报表</t>
   </si>
   <si>
-    <t>Monthly Report</t>
-  </si>
-  <si>
-    <t>月次レポート</t>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>月次</t>
   </si>
   <si>
     <t>LC_YEAR_REPORT</t>
@@ -481,10 +481,10 @@
     <t>年报表</t>
   </si>
   <si>
-    <t>Yearly Report</t>
-  </si>
-  <si>
-    <t>年次レポート</t>
+    <t>Yearly</t>
+  </si>
+  <si>
+    <t>年次</t>
   </si>
   <si>
     <t>LC_FIRST_HALF</t>
@@ -493,10 +493,10 @@
     <t>上半月</t>
   </si>
   <si>
-    <t>First Half of the Month</t>
-  </si>
-  <si>
-    <t>月の前半</t>
+    <t>1st Half</t>
+  </si>
+  <si>
+    <t>前半</t>
   </si>
   <si>
     <t>LC_SECOND_HALF</t>
@@ -505,10 +505,10 @@
     <t>下半月</t>
   </si>
   <si>
-    <t>Second Half of the Month</t>
-  </si>
-  <si>
-    <t>月の後半</t>
+    <t>2nd Half</t>
+  </si>
+  <si>
+    <t>後半</t>
   </si>
   <si>
     <t>LC_MONTH_TOP</t>

</xml_diff>

<commit_message>
feat: modify category detail
</commit_message>
<xml_diff>
--- a/src/locales/moneyGone.xlsx
+++ b/src/locales/moneyGone.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="485">
   <si>
     <t>key</t>
   </si>
@@ -1451,6 +1451,21 @@
   </si>
   <si>
     <t>削除</t>
+  </si>
+  <si>
+    <t>LC_PREVIEW</t>
+  </si>
+  <si>
+    <t>預覽</t>
+  </si>
+  <si>
+    <t>预览</t>
+  </si>
+  <si>
+    <t>Preview</t>
+  </si>
+  <si>
+    <t>プレビュー</t>
   </si>
 </sst>
 </file>
@@ -3471,6 +3486,23 @@
         <v>479</v>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>484</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: modify api message
</commit_message>
<xml_diff>
--- a/src/locales/moneyGone.xlsx
+++ b/src/locales/moneyGone.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="490">
   <si>
     <t>key</t>
   </si>
@@ -427,6 +427,21 @@
     <t>今月はまだ支出がありません</t>
   </si>
   <si>
+    <t>LC_SEARCH_EMPTY</t>
+  </si>
+  <si>
+    <t>沒有符合搜尋的項目</t>
+  </si>
+  <si>
+    <t>没有符合搜索的项目</t>
+  </si>
+  <si>
+    <t>No matching results</t>
+  </si>
+  <si>
+    <t>一致する項目がありません</t>
+  </si>
+  <si>
     <t>LC_BAR_CHART</t>
   </si>
   <si>
@@ -958,6 +973,21 @@
     <t>ショートカット {name} を削除してもよろしいですか？</t>
   </si>
   <si>
+    <t>LC_PREVIEW</t>
+  </si>
+  <si>
+    <t>預覽</t>
+  </si>
+  <si>
+    <t>预览</t>
+  </si>
+  <si>
+    <t>Preview</t>
+  </si>
+  <si>
+    <t>プレビュー</t>
+  </si>
+  <si>
     <t>LC_LOGIN</t>
   </si>
   <si>
@@ -1451,21 +1481,6 @@
   </si>
   <si>
     <t>削除</t>
-  </si>
-  <si>
-    <t>LC_PREVIEW</t>
-  </si>
-  <si>
-    <t>預覽</t>
-  </si>
-  <si>
-    <t>预览</t>
-  </si>
-  <si>
-    <t>Preview</t>
-  </si>
-  <si>
-    <t>プレビュー</t>
   </si>
 </sst>
 </file>
@@ -2241,28 +2256,28 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
+      <c r="A33" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>142</v>
-      </c>
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
@@ -2323,38 +2338,38 @@
         <v>159</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>168</v>
@@ -2452,28 +2467,28 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
+      <c r="A46" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>200</v>
-      </c>
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
@@ -2602,21 +2617,21 @@
         <v>237</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>242</v>
@@ -2867,45 +2882,45 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
+      <c r="A71" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>324</v>
-      </c>
+      <c r="A73" s="1"/>
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
@@ -3061,45 +3076,45 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1"/>
-      <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1"/>
+      <c r="A83" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>377</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>379</v>
-      </c>
+      <c r="A85" s="1"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="s">
@@ -3204,86 +3219,86 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1"/>
-      <c r="B92" s="1"/>
-      <c r="C92" s="1"/>
-      <c r="D92" s="1"/>
-      <c r="E92" s="1"/>
+      <c r="A92" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>414</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="E94" s="1" t="s">
-        <v>419</v>
-      </c>
+      <c r="A94" s="1"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
     </row>
     <row r="95">
-      <c r="A95" s="1"/>
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-      <c r="D95" s="1"/>
-      <c r="E95" s="1"/>
+      <c r="A95" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>424</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>429</v>
-      </c>
+      <c r="A97" s="1"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="s">
@@ -3303,45 +3318,45 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1"/>
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
-      <c r="E99" s="1"/>
+      <c r="A99" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D101" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="E101" s="1" t="s">
-        <v>444</v>
-      </c>
+      <c r="A101" s="1"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="s">
@@ -3351,85 +3366,85 @@
         <v>446</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1"/>
-      <c r="B104" s="1"/>
-      <c r="C104" s="1"/>
-      <c r="D104" s="1"/>
-      <c r="E104" s="1"/>
+      <c r="A104" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>458</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="E106" s="1" t="s">
-        <v>460</v>
-      </c>
+      <c r="A106" s="1"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>464</v>
@@ -3437,27 +3452,27 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>472</v>
@@ -3501,6 +3516,23 @@
       </c>
       <c r="E111" s="1" t="s">
         <v>484</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>